<commit_message>
Atualiza financas.xlsx - 072026 - 25/07/2026
</commit_message>
<xml_diff>
--- a/financas.xlsx
+++ b/financas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/fea781441e4f247c/Documentos/Finanças/2026/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="362" documentId="8_{B7224BD9-7546-4D39-AD24-E9DCD61BD67B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78543C44-ABD6-4823-8F6D-B177A98B3AB2}"/>
+  <xr:revisionPtr revIDLastSave="440" documentId="8_{B7224BD9-7546-4D39-AD24-E9DCD61BD67B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{09D21FCF-1DF7-421D-AC92-8322B8783B7C}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Saldo" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="243">
   <si>
     <t>Valor para o mês</t>
   </si>
@@ -414,15 +414,42 @@
     <t>Serviço de nuvem da câmera</t>
   </si>
   <si>
+    <t>Rappi</t>
+  </si>
+  <si>
     <t>Gasolina</t>
   </si>
   <si>
-    <t>Rappi</t>
-  </si>
-  <si>
     <t>Lanche</t>
   </si>
   <si>
+    <t>Gibis</t>
+  </si>
+  <si>
+    <t>Bonffas Beer</t>
+  </si>
+  <si>
+    <t>Gasolina Pirassunusng</t>
+  </si>
+  <si>
+    <t>Hot Wheels</t>
+  </si>
+  <si>
+    <t>Pagamento Hot Wheels</t>
+  </si>
+  <si>
+    <t>Kikão</t>
+  </si>
+  <si>
+    <t>Gasolina de Volta</t>
+  </si>
+  <si>
+    <t>Odisseia</t>
+  </si>
+  <si>
+    <t>Pagamento Odisseia</t>
+  </si>
+  <si>
     <t>Vivo</t>
   </si>
   <si>
@@ -618,6 +645,12 @@
     <t>Pagamento Edilson</t>
   </si>
   <si>
+    <t>Dinheiro Nano</t>
+  </si>
+  <si>
+    <t>Recolhimento Receita</t>
+  </si>
+  <si>
     <t>Ilumeo Julho - 1º PPT</t>
   </si>
   <si>
@@ -717,37 +750,31 @@
     <t>Dera</t>
   </si>
   <si>
-    <t>Gibis</t>
-  </si>
-  <si>
-    <t>Bonffas Beer</t>
-  </si>
-  <si>
-    <t>Gasolina Pirassunusng</t>
-  </si>
-  <si>
-    <t>Hot Wheels</t>
-  </si>
-  <si>
-    <t>Pagamento Hot Wheels</t>
-  </si>
-  <si>
-    <t>Kikão</t>
-  </si>
-  <si>
-    <t>Gasolina de Volta</t>
-  </si>
-  <si>
-    <t>Odisseia</t>
-  </si>
-  <si>
-    <t>Pagamento Odisseia</t>
-  </si>
-  <si>
-    <t>Dinheiro Nano</t>
-  </si>
-  <si>
-    <t>Recolhimento Receita</t>
+    <t>Ifood</t>
+  </si>
+  <si>
+    <t>Mercado</t>
+  </si>
+  <si>
+    <t>Rappi 1</t>
+  </si>
+  <si>
+    <t>Rappi 2</t>
+  </si>
+  <si>
+    <t>Saco de lixo e copo descartável</t>
+  </si>
+  <si>
+    <t>Mr Jones</t>
+  </si>
+  <si>
+    <t>Renner - Presente Stella</t>
+  </si>
+  <si>
+    <t>Renner Stella</t>
+  </si>
+  <si>
+    <t>Baked Potato</t>
   </si>
 </sst>
 </file>
@@ -1232,20 +1259,20 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="16">
+  <dxfs count="15">
     <dxf>
       <font>
         <color rgb="FFFF0000"/>
@@ -1320,14 +1347,6 @@
       <fill>
         <patternFill>
           <bgColor theme="7" tint="0.79989013336588644"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFD9E1F2"/>
-          <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1661,7 +1680,7 @@
   <sheetData>
     <row r="1" spans="2:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:6" ht="23.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="77" t="s">
+      <c r="B2" s="75" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -1673,15 +1692,15 @@
       </c>
     </row>
     <row r="3" spans="2:6" ht="24" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="78"/>
+      <c r="B3" s="76"/>
       <c r="C3" s="6">
         <f>C5-C8-C10-C11-C22+C23+C7</f>
-        <v>1732.8714047619037</v>
+        <v>2098.2464047619037</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="6">
         <f>E5-E8-E10-E11-E22+E23</f>
-        <v>3729.3575000000001</v>
+        <v>3520.8625000000011</v>
       </c>
     </row>
     <row r="4" spans="2:6" ht="7.5" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1690,7 +1709,7 @@
         <v>3</v>
       </c>
       <c r="C5" s="8">
-        <v>10000</v>
+        <v>10200</v>
       </c>
       <c r="D5" s="9"/>
       <c r="E5" s="8">
@@ -1703,12 +1722,12 @@
       </c>
       <c r="C6" s="8">
         <f>-SUM(C8,C10,C11)</f>
-        <v>-7605.1285952380968</v>
+        <v>-7939.7535952380968</v>
       </c>
       <c r="D6" s="9"/>
       <c r="E6" s="8">
         <f>-SUM(E8,E10,E11)</f>
-        <v>-5270.6424999999999</v>
+        <v>-5479.1374999999998</v>
       </c>
     </row>
     <row r="7" spans="2:6" x14ac:dyDescent="0.25">
@@ -1739,12 +1758,12 @@
       </c>
       <c r="C9" s="8">
         <f>NuBank!E2</f>
-        <v>5182.8969285714293</v>
+        <v>5517.5219285714293</v>
       </c>
       <c r="D9" s="9"/>
       <c r="E9" s="8">
         <f>NuBank!F2</f>
-        <v>1888.5724999999998</v>
+        <v>2097.0674999999997</v>
       </c>
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.25">
@@ -1753,12 +1772,12 @@
       </c>
       <c r="C10" s="11">
         <f>'Compensasões e Transferências'!D4</f>
-        <v>5182.8969285714293</v>
+        <v>5517.5219285714293</v>
       </c>
       <c r="D10" s="12"/>
       <c r="E10" s="11">
         <f>'Compensasões e Transferências'!C4</f>
-        <v>1888.5724999999998</v>
+        <v>2097.0674999999997</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.25">
@@ -1895,7 +1914,7 @@
         <v>18</v>
       </c>
       <c r="C22" s="8">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="D22" s="9"/>
       <c r="E22" s="8">
@@ -2131,11 +2150,11 @@
       </c>
       <c r="C4" s="8">
         <f>Saldo!E9+C5</f>
-        <v>1888.5724999999998</v>
+        <v>2097.0674999999997</v>
       </c>
       <c r="D4" s="27">
         <f>Saldo!C9+D5</f>
-        <v>5182.8969285714293</v>
+        <v>5517.5219285714293</v>
       </c>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.25">
@@ -2239,7 +2258,7 @@
       </c>
       <c r="C17" s="11">
         <f>SUM(C3,C4,C5,C10)</f>
-        <v>3936.2574999999997</v>
+        <v>4144.7524999999996</v>
       </c>
       <c r="D17" s="30"/>
     </row>
@@ -3012,15 +3031,15 @@
     <row r="2" spans="3:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D2" s="48">
         <f>SUM(L6:L377)</f>
-        <v>7121.4694285714277</v>
+        <v>7681.5594285714278</v>
       </c>
       <c r="E2" s="35">
         <f>SUMIF($E$6:$E$377,E1,$M$6:$M$377)</f>
-        <v>5182.8969285714293</v>
+        <v>5517.5219285714293</v>
       </c>
       <c r="F2" s="35">
         <f>SUMIF($F$6:$F$377,F1,$M$6:$M$377)</f>
-        <v>1888.5724999999998</v>
+        <v>2097.0674999999997</v>
       </c>
       <c r="G2" s="35">
         <f>SUMIF($G$6:$G$377,G1,$M$6:$M$377)</f>
@@ -5741,7 +5760,7 @@
     <row r="65" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C65" s="38"/>
       <c r="D65" s="49" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E65" s="40" t="s">
         <v>1</v>
@@ -5783,7 +5802,7 @@
     <row r="66" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C66" s="38"/>
       <c r="D66" s="49" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E66" s="40"/>
       <c r="F66" s="40" t="s">
@@ -5823,7 +5842,7 @@
     <row r="67" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C67" s="38"/>
       <c r="D67" s="49" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E67" s="40" t="s">
         <v>1</v>
@@ -5903,7 +5922,7 @@
     <row r="69" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C69" s="38"/>
       <c r="D69" s="49" t="s">
-        <v>223</v>
+        <v>125</v>
       </c>
       <c r="E69" s="40" t="s">
         <v>1</v>
@@ -5943,7 +5962,7 @@
     <row r="70" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C70" s="38"/>
       <c r="D70" s="49" t="s">
-        <v>224</v>
+        <v>126</v>
       </c>
       <c r="E70" s="40" t="s">
         <v>1</v>
@@ -5983,7 +6002,7 @@
     <row r="71" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C71" s="38"/>
       <c r="D71" s="49" t="s">
-        <v>225</v>
+        <v>127</v>
       </c>
       <c r="E71" s="40" t="s">
         <v>1</v>
@@ -6025,7 +6044,7 @@
     <row r="72" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C72" s="38"/>
       <c r="D72" s="49" t="s">
-        <v>226</v>
+        <v>128</v>
       </c>
       <c r="E72" s="40" t="s">
         <v>1</v>
@@ -6065,7 +6084,7 @@
     <row r="73" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C73" s="38"/>
       <c r="D73" s="49" t="s">
-        <v>227</v>
+        <v>129</v>
       </c>
       <c r="E73" s="40" t="s">
         <v>1</v>
@@ -6105,7 +6124,7 @@
     <row r="74" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C74" s="38"/>
       <c r="D74" s="49" t="s">
-        <v>228</v>
+        <v>130</v>
       </c>
       <c r="E74" s="40" t="s">
         <v>1</v>
@@ -6147,7 +6166,7 @@
     <row r="75" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C75" s="38"/>
       <c r="D75" s="49" t="s">
-        <v>229</v>
+        <v>131</v>
       </c>
       <c r="E75" s="40"/>
       <c r="F75" s="40" t="s">
@@ -6187,7 +6206,7 @@
     <row r="76" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C76" s="38"/>
       <c r="D76" s="49" t="s">
-        <v>230</v>
+        <v>132</v>
       </c>
       <c r="E76" s="40" t="s">
         <v>1</v>
@@ -6229,7 +6248,7 @@
     <row r="77" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C77" s="38"/>
       <c r="D77" s="49" t="s">
-        <v>231</v>
+        <v>133</v>
       </c>
       <c r="E77" s="40" t="s">
         <v>1</v>
@@ -6268,24 +6287,32 @@
     </row>
     <row r="78" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C78" s="38"/>
-      <c r="D78" s="49"/>
-      <c r="E78" s="40"/>
-      <c r="F78" s="40"/>
+      <c r="D78" s="49" t="s">
+        <v>234</v>
+      </c>
+      <c r="E78" s="40" t="s">
+        <v>1</v>
+      </c>
+      <c r="F78" s="40" t="s">
+        <v>2</v>
+      </c>
       <c r="G78" s="40"/>
       <c r="H78" s="40">
         <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="I78" s="41"/>
+        <v>2</v>
+      </c>
+      <c r="I78" s="41">
+        <v>79</v>
+      </c>
       <c r="J78" s="41"/>
       <c r="K78" s="41"/>
       <c r="L78" s="41">
         <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="M78" s="41" t="str">
+        <v>79</v>
+      </c>
+      <c r="M78" s="41">
         <f t="shared" si="13"/>
-        <v/>
+        <v>39.5</v>
       </c>
       <c r="N78" s="42">
         <v>1</v>
@@ -6302,24 +6329,32 @@
     </row>
     <row r="79" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C79" s="38"/>
-      <c r="D79" s="49"/>
-      <c r="E79" s="40"/>
-      <c r="F79" s="40"/>
+      <c r="D79" s="49" t="s">
+        <v>235</v>
+      </c>
+      <c r="E79" s="40" t="s">
+        <v>1</v>
+      </c>
+      <c r="F79" s="40" t="s">
+        <v>2</v>
+      </c>
       <c r="G79" s="40"/>
       <c r="H79" s="40">
         <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="I79" s="41"/>
+        <v>2</v>
+      </c>
+      <c r="I79" s="41">
+        <v>56.27</v>
+      </c>
       <c r="J79" s="41"/>
       <c r="K79" s="41"/>
       <c r="L79" s="41">
         <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="M79" s="41" t="str">
+        <v>56.27</v>
+      </c>
+      <c r="M79" s="41">
         <f t="shared" si="13"/>
-        <v/>
+        <v>28.135000000000002</v>
       </c>
       <c r="N79" s="42">
         <v>1</v>
@@ -6336,24 +6371,32 @@
     </row>
     <row r="80" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C80" s="38"/>
-      <c r="D80" s="49"/>
-      <c r="E80" s="40"/>
-      <c r="F80" s="40"/>
+      <c r="D80" s="49" t="s">
+        <v>236</v>
+      </c>
+      <c r="E80" s="40" t="s">
+        <v>1</v>
+      </c>
+      <c r="F80" s="40" t="s">
+        <v>2</v>
+      </c>
       <c r="G80" s="40"/>
       <c r="H80" s="40">
         <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="I80" s="41"/>
+        <v>2</v>
+      </c>
+      <c r="I80" s="41">
+        <v>82.49</v>
+      </c>
       <c r="J80" s="41"/>
       <c r="K80" s="41"/>
       <c r="L80" s="41">
         <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="M80" s="41" t="str">
+        <v>82.49</v>
+      </c>
+      <c r="M80" s="41">
         <f t="shared" si="13"/>
-        <v/>
+        <v>41.244999999999997</v>
       </c>
       <c r="N80" s="42">
         <v>1</v>
@@ -6370,24 +6413,32 @@
     </row>
     <row r="81" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C81" s="38"/>
-      <c r="D81" s="49"/>
-      <c r="E81" s="40"/>
-      <c r="F81" s="40"/>
+      <c r="D81" s="49" t="s">
+        <v>237</v>
+      </c>
+      <c r="E81" s="40" t="s">
+        <v>1</v>
+      </c>
+      <c r="F81" s="40" t="s">
+        <v>2</v>
+      </c>
       <c r="G81" s="40"/>
       <c r="H81" s="40">
         <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="I81" s="41"/>
+        <v>2</v>
+      </c>
+      <c r="I81" s="41">
+        <v>49.91</v>
+      </c>
       <c r="J81" s="41"/>
       <c r="K81" s="41"/>
       <c r="L81" s="41">
         <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="M81" s="41" t="str">
+        <v>49.91</v>
+      </c>
+      <c r="M81" s="41">
         <f t="shared" si="13"/>
-        <v/>
+        <v>24.954999999999998</v>
       </c>
       <c r="N81" s="42">
         <v>1</v>
@@ -6404,24 +6455,32 @@
     </row>
     <row r="82" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C82" s="38"/>
-      <c r="D82" s="49"/>
-      <c r="E82" s="40"/>
-      <c r="F82" s="40"/>
+      <c r="D82" s="49" t="s">
+        <v>238</v>
+      </c>
+      <c r="E82" s="40" t="s">
+        <v>1</v>
+      </c>
+      <c r="F82" s="40" t="s">
+        <v>2</v>
+      </c>
       <c r="G82" s="40"/>
       <c r="H82" s="40">
         <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="I82" s="41"/>
+        <v>2</v>
+      </c>
+      <c r="I82" s="41">
+        <v>41.5</v>
+      </c>
       <c r="J82" s="41"/>
       <c r="K82" s="41"/>
       <c r="L82" s="41">
         <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="M82" s="41" t="str">
+        <v>41.5</v>
+      </c>
+      <c r="M82" s="41">
         <f t="shared" si="13"/>
-        <v/>
+        <v>20.75</v>
       </c>
       <c r="N82" s="42">
         <v>1</v>
@@ -6438,24 +6497,30 @@
     </row>
     <row r="83" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C83" s="38"/>
-      <c r="D83" s="49"/>
-      <c r="E83" s="40"/>
+      <c r="D83" s="49" t="s">
+        <v>239</v>
+      </c>
+      <c r="E83" s="40" t="s">
+        <v>1</v>
+      </c>
       <c r="F83" s="40"/>
       <c r="G83" s="40"/>
       <c r="H83" s="40">
         <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="I83" s="41"/>
+        <v>1</v>
+      </c>
+      <c r="I83" s="41">
+        <v>106.04</v>
+      </c>
       <c r="J83" s="41"/>
       <c r="K83" s="41"/>
       <c r="L83" s="41">
         <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="M83" s="41" t="str">
+        <v>106.04</v>
+      </c>
+      <c r="M83" s="41">
         <f t="shared" si="13"/>
-        <v/>
+        <v>106.04</v>
       </c>
       <c r="N83" s="42">
         <v>1</v>
@@ -6472,7 +6537,9 @@
     </row>
     <row r="84" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C84" s="38"/>
-      <c r="D84" s="49"/>
+      <c r="D84" s="49" t="s">
+        <v>119</v>
+      </c>
       <c r="E84" s="40"/>
       <c r="F84" s="40"/>
       <c r="G84" s="40"/>
@@ -6480,12 +6547,14 @@
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="I84" s="41"/>
+      <c r="I84" s="41">
+        <v>16.97</v>
+      </c>
       <c r="J84" s="41"/>
       <c r="K84" s="41"/>
       <c r="L84" s="41">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>16.97</v>
       </c>
       <c r="M84" s="41" t="str">
         <f t="shared" si="13"/>
@@ -6506,32 +6575,42 @@
     </row>
     <row r="85" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C85" s="38"/>
-      <c r="D85" s="49"/>
-      <c r="E85" s="40"/>
+      <c r="D85" s="49" t="s">
+        <v>240</v>
+      </c>
+      <c r="E85" s="40" t="s">
+        <v>1</v>
+      </c>
       <c r="F85" s="40"/>
       <c r="G85" s="40"/>
       <c r="H85" s="40">
         <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="I85" s="41"/>
-      <c r="J85" s="41"/>
+        <v>1</v>
+      </c>
+      <c r="I85" s="41">
+        <v>72</v>
+      </c>
+      <c r="J85" s="41" t="s">
+        <v>44</v>
+      </c>
       <c r="K85" s="41"/>
       <c r="L85" s="41">
         <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="M85" s="41" t="str">
+        <v>24</v>
+      </c>
+      <c r="M85" s="41">
         <f t="shared" si="13"/>
-        <v/>
+        <v>24</v>
       </c>
       <c r="N85" s="42">
-        <v>1</v>
-      </c>
-      <c r="O85" s="38"/>
-      <c r="P85" s="38" t="str">
+        <v>3</v>
+      </c>
+      <c r="O85" s="67">
+        <v>46240</v>
+      </c>
+      <c r="P85" s="67">
         <f t="shared" si="14"/>
-        <v/>
+        <v>46301</v>
       </c>
       <c r="Q85" s="40" t="str">
         <f t="shared" ca="1" si="15"/>
@@ -6540,32 +6619,42 @@
     </row>
     <row r="86" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C86" s="38"/>
-      <c r="D86" s="49"/>
+      <c r="D86" s="49" t="s">
+        <v>241</v>
+      </c>
       <c r="E86" s="40"/>
-      <c r="F86" s="40"/>
+      <c r="F86" s="40" t="s">
+        <v>2</v>
+      </c>
       <c r="G86" s="40"/>
       <c r="H86" s="40">
         <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="I86" s="41"/>
-      <c r="J86" s="41"/>
+        <v>1</v>
+      </c>
+      <c r="I86" s="41">
+        <v>161.72999999999999</v>
+      </c>
+      <c r="J86" s="41" t="s">
+        <v>44</v>
+      </c>
       <c r="K86" s="41"/>
       <c r="L86" s="41">
         <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="M86" s="41" t="str">
+        <v>53.91</v>
+      </c>
+      <c r="M86" s="41">
         <f t="shared" si="13"/>
-        <v/>
+        <v>53.91</v>
       </c>
       <c r="N86" s="42">
-        <v>1</v>
-      </c>
-      <c r="O86" s="38"/>
-      <c r="P86" s="38" t="str">
+        <v>3</v>
+      </c>
+      <c r="O86" s="67">
+        <v>46240</v>
+      </c>
+      <c r="P86" s="67">
         <f t="shared" si="14"/>
-        <v/>
+        <v>46301</v>
       </c>
       <c r="Q86" s="40" t="str">
         <f t="shared" ca="1" si="15"/>
@@ -6574,24 +6663,30 @@
     </row>
     <row r="87" spans="3:17" x14ac:dyDescent="0.25">
       <c r="C87" s="38"/>
-      <c r="D87" s="49"/>
-      <c r="E87" s="40"/>
+      <c r="D87" s="49" t="s">
+        <v>242</v>
+      </c>
+      <c r="E87" s="40" t="s">
+        <v>1</v>
+      </c>
       <c r="F87" s="40"/>
       <c r="G87" s="40"/>
       <c r="H87" s="40">
         <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="I87" s="41"/>
+        <v>1</v>
+      </c>
+      <c r="I87" s="41">
+        <v>50</v>
+      </c>
       <c r="J87" s="41"/>
       <c r="K87" s="41"/>
       <c r="L87" s="41">
         <f t="shared" si="12"/>
-        <v>0</v>
-      </c>
-      <c r="M87" s="41" t="str">
+        <v>50</v>
+      </c>
+      <c r="M87" s="41">
         <f t="shared" si="13"/>
-        <v/>
+        <v>50</v>
       </c>
       <c r="N87" s="42">
         <v>1</v>
@@ -8734,7 +8829,7 @@
   </sheetData>
   <autoFilter ref="C5:Q150" xr:uid="{00000000-0009-0000-0000-000003000000}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C6:Q150">
-      <sortCondition sortBy="cellColor" ref="J5:J150" dxfId="15"/>
+      <sortCondition sortBy="cellColor" ref="J5:J150" dxfId="14"/>
     </sortState>
   </autoFilter>
   <conditionalFormatting sqref="I6:I150">
@@ -8851,7 +8946,7 @@
     </row>
     <row r="4" spans="2:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D4" s="58" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="E4" s="59" t="s">
         <v>1</v>
@@ -8892,7 +8987,7 @@
         <v>1</v>
       </c>
       <c r="D5" s="57" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="E5" s="39" t="s">
         <v>1</v>
@@ -8934,7 +9029,7 @@
         <v>2382.0700000000002</v>
       </c>
       <c r="D6" s="57" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="E6" s="39" t="s">
         <v>1</v>
@@ -8972,7 +9067,7 @@
     <row r="7" spans="2:18" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="63"/>
       <c r="D7" s="57" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="E7" s="39" t="s">
         <v>1</v>
@@ -9053,7 +9148,7 @@
         <v>3382.07</v>
       </c>
       <c r="D9" s="57" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="E9" s="39" t="s">
         <v>1</v>
@@ -9091,7 +9186,7 @@
     </row>
     <row r="10" spans="2:18" x14ac:dyDescent="0.25">
       <c r="D10" s="57" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="E10" s="39"/>
       <c r="F10" s="40" t="s">
@@ -9292,7 +9387,7 @@
     <row r="1" spans="2:15" x14ac:dyDescent="0.25">
       <c r="G1" s="2"/>
       <c r="N1" s="50" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" spans="2:15" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -9302,10 +9397,10 @@
     <row r="3" spans="2:15" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="G3" s="2"/>
       <c r="L3" s="50" t="s">
-        <v>132</v>
-      </c>
-      <c r="M3" s="75" t="s">
-        <v>133</v>
+        <v>141</v>
+      </c>
+      <c r="M3" s="77" t="s">
+        <v>142</v>
       </c>
       <c r="N3" s="46">
         <f>SUM(N5:N21)</f>
@@ -9316,9 +9411,9 @@
     <row r="4" spans="2:15" x14ac:dyDescent="0.25">
       <c r="G4" s="2"/>
       <c r="L4" s="51" t="s">
-        <v>134</v>
-      </c>
-      <c r="M4" s="76"/>
+        <v>143</v>
+      </c>
+      <c r="M4" s="78"/>
       <c r="N4" s="52"/>
     </row>
     <row r="5" spans="2:15" x14ac:dyDescent="0.25">
@@ -9327,7 +9422,7 @@
       <c r="F5" s="16"/>
       <c r="G5" s="31"/>
       <c r="L5" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="N5" s="1">
         <v>4912</v>
@@ -9337,7 +9432,7 @@
     <row r="6" spans="2:15" x14ac:dyDescent="0.25">
       <c r="G6" s="2"/>
       <c r="L6" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="N6" s="1">
         <v>101</v>
@@ -9351,10 +9446,10 @@
       <c r="F8" s="16"/>
       <c r="G8" s="53"/>
       <c r="L8" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="M8" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="N8" s="1">
         <v>338</v>
@@ -9362,41 +9457,41 @@
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.25">
       <c r="F9" s="50" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="G9" s="31"/>
       <c r="N9" s="46"/>
     </row>
     <row r="10" spans="2:15" x14ac:dyDescent="0.25">
       <c r="E10" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="F10" s="16">
         <f>SUM(G11:I11)</f>
-        <v>164.15000000000146</v>
+        <v>4597.1500000000015</v>
       </c>
       <c r="G10" s="54" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="H10" s="54" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="I10" s="54" t="s">
-        <v>143</v>
+        <v>152</v>
       </c>
       <c r="N10" s="46"/>
     </row>
     <row r="11" spans="2:15" x14ac:dyDescent="0.25">
       <c r="E11" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="F11" s="16">
         <f>SUM(G11:H11)</f>
-        <v>164.15000000000146</v>
+        <v>4597.1500000000015</v>
       </c>
       <c r="G11" s="1">
         <f>G12+SUM(G14:G496)</f>
-        <v>164.15000000000146</v>
+        <v>4597.1500000000015</v>
       </c>
       <c r="H11" s="1">
         <f>H12+SUM(H14:H496)</f>
@@ -9410,7 +9505,7 @@
     </row>
     <row r="12" spans="2:15" x14ac:dyDescent="0.25">
       <c r="F12" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="G12" s="1">
         <v>15250</v>
@@ -9419,7 +9514,7 @@
     </row>
     <row r="13" spans="2:15" x14ac:dyDescent="0.25">
       <c r="F13" s="74" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="G13" s="55"/>
       <c r="H13" s="74"/>
@@ -9430,7 +9525,7 @@
       <c r="C14" s="56"/>
       <c r="D14" s="56"/>
       <c r="F14" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="G14" s="56"/>
       <c r="H14" s="56"/>
@@ -9441,7 +9536,7 @@
       <c r="C15" s="56"/>
       <c r="D15" s="56"/>
       <c r="F15" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="G15" s="56">
         <v>773.35</v>
@@ -9454,7 +9549,7 @@
       <c r="C16" s="56"/>
       <c r="D16" s="56"/>
       <c r="F16" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="G16" s="56">
         <v>-5148</v>
@@ -9467,7 +9562,7 @@
       <c r="C17" s="56"/>
       <c r="D17" s="56"/>
       <c r="F17" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="G17" s="56">
         <v>-168</v>
@@ -9480,7 +9575,7 @@
       <c r="C18" s="56"/>
       <c r="D18" s="56"/>
       <c r="F18" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="G18" s="56">
         <v>-1700</v>
@@ -9493,7 +9588,7 @@
       <c r="C19" s="56"/>
       <c r="D19" s="56"/>
       <c r="F19" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="G19" s="56">
         <v>5148</v>
@@ -9506,7 +9601,7 @@
       <c r="C20" s="56"/>
       <c r="D20" s="56"/>
       <c r="F20" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="G20" s="56">
         <v>-4938</v>
@@ -9519,7 +9614,7 @@
       <c r="C21" s="56"/>
       <c r="D21" s="56"/>
       <c r="F21" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="G21" s="56">
         <v>-1595</v>
@@ -9532,7 +9627,7 @@
       <c r="C22" s="56"/>
       <c r="D22" s="56"/>
       <c r="F22" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="G22" s="56">
         <v>-4677</v>
@@ -9545,7 +9640,7 @@
       <c r="C23" s="56"/>
       <c r="D23" s="56"/>
       <c r="F23" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="G23" s="56">
         <v>-200</v>
@@ -9558,7 +9653,7 @@
       <c r="C24" s="56"/>
       <c r="D24" s="56"/>
       <c r="F24" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="G24" s="56">
         <v>4677</v>
@@ -9571,7 +9666,7 @@
       <c r="C25" s="56"/>
       <c r="D25" s="56"/>
       <c r="F25" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="G25" s="56">
         <v>-750</v>
@@ -9584,7 +9679,7 @@
       <c r="C26" s="56"/>
       <c r="D26" s="56"/>
       <c r="F26" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="G26" s="56">
         <v>-652</v>
@@ -9597,7 +9692,7 @@
       <c r="C27" s="56"/>
       <c r="D27" s="56"/>
       <c r="F27" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="G27" s="56">
         <v>11100</v>
@@ -9610,7 +9705,7 @@
       <c r="C28" s="56"/>
       <c r="D28" s="56"/>
       <c r="F28" t="s">
-        <v>158</v>
+        <v>167</v>
       </c>
       <c r="G28" s="56">
         <v>-396</v>
@@ -9623,7 +9718,7 @@
       <c r="C29" s="56"/>
       <c r="D29" s="56"/>
       <c r="F29" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="G29" s="56">
         <v>-4211</v>
@@ -9636,7 +9731,7 @@
       <c r="C30" s="56"/>
       <c r="D30" s="56"/>
       <c r="F30" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="G30" s="56">
         <v>-450</v>
@@ -9649,7 +9744,7 @@
       <c r="C31" s="56"/>
       <c r="D31" s="56"/>
       <c r="F31" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="G31" s="56">
         <v>-1197</v>
@@ -9675,7 +9770,7 @@
       <c r="C33" s="56"/>
       <c r="D33" s="56"/>
       <c r="F33" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
       <c r="G33" s="56">
         <v>-830</v>
@@ -9688,7 +9783,7 @@
       <c r="C34" s="56"/>
       <c r="D34" s="56"/>
       <c r="F34" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="G34" s="56">
         <v>4211</v>
@@ -9701,7 +9796,7 @@
       <c r="C35" s="56"/>
       <c r="D35" s="56"/>
       <c r="F35" t="s">
-        <v>163</v>
+        <v>172</v>
       </c>
       <c r="G35" s="56">
         <v>-200</v>
@@ -9714,7 +9809,7 @@
       <c r="C36" s="56"/>
       <c r="D36" s="56"/>
       <c r="F36" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="G36" s="56">
         <v>10000</v>
@@ -9727,7 +9822,7 @@
       <c r="C37" s="56"/>
       <c r="D37" s="56"/>
       <c r="F37" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="G37" s="56">
         <v>-200</v>
@@ -9740,7 +9835,7 @@
       <c r="C38" s="56"/>
       <c r="D38" s="56"/>
       <c r="F38" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="G38" s="56">
         <v>-381</v>
@@ -9753,7 +9848,7 @@
       <c r="C39" s="56"/>
       <c r="D39" s="56"/>
       <c r="F39" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="G39" s="56">
         <v>-4911</v>
@@ -9767,7 +9862,7 @@
       <c r="D40" s="56"/>
       <c r="E40" s="2"/>
       <c r="F40" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="G40" s="56">
         <v>-5700</v>
@@ -9780,7 +9875,7 @@
       <c r="C41" s="56"/>
       <c r="D41" s="56"/>
       <c r="F41" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="G41" s="56">
         <v>-400</v>
@@ -9793,7 +9888,7 @@
       <c r="C42" s="56"/>
       <c r="D42" s="56"/>
       <c r="F42" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="G42" s="56">
         <v>-450</v>
@@ -9806,7 +9901,7 @@
       <c r="C43" s="56"/>
       <c r="D43" s="56"/>
       <c r="F43" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="G43" s="56">
         <v>-640</v>
@@ -9820,7 +9915,7 @@
       <c r="D44" s="56"/>
       <c r="E44" s="2"/>
       <c r="F44" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="G44" s="56">
         <v>5700</v>
@@ -9833,7 +9928,7 @@
       <c r="C45" s="56"/>
       <c r="D45" s="56"/>
       <c r="F45" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
       <c r="G45" s="56">
         <v>-130</v>
@@ -9846,7 +9941,7 @@
       <c r="C46" s="56"/>
       <c r="D46" s="56"/>
       <c r="F46" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
       <c r="G46" s="56">
         <v>-250</v>
@@ -9859,7 +9954,7 @@
       <c r="C47" s="56"/>
       <c r="D47" s="56"/>
       <c r="F47" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="G47" s="56">
         <v>-112.2</v>
@@ -9872,7 +9967,7 @@
       <c r="C48" s="56"/>
       <c r="D48" s="56"/>
       <c r="F48" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="G48" s="56">
         <v>4911</v>
@@ -9885,7 +9980,7 @@
       <c r="C49" s="56"/>
       <c r="D49" s="56"/>
       <c r="F49" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
       <c r="G49" s="56">
         <v>-3000</v>
@@ -9898,7 +9993,7 @@
       <c r="C50" s="56"/>
       <c r="D50" s="56"/>
       <c r="F50" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="G50" s="56">
         <v>-4000</v>
@@ -9911,7 +10006,7 @@
       <c r="C51" s="56"/>
       <c r="D51" s="56"/>
       <c r="F51" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="G51" s="56">
         <v>-200</v>
@@ -9924,7 +10019,7 @@
       <c r="C52" s="56"/>
       <c r="D52" s="56"/>
       <c r="F52" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="G52" s="56">
         <v>-4612</v>
@@ -9935,7 +10030,7 @@
     </row>
     <row r="53" spans="3:14" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="F53" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
       <c r="G53" s="56">
         <v>-700</v>
@@ -9946,7 +10041,7 @@
     </row>
     <row r="54" spans="3:14" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="F54" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G54" s="56">
         <v>-880</v>
@@ -9957,7 +10052,7 @@
     </row>
     <row r="55" spans="3:14" outlineLevel="1" x14ac:dyDescent="0.25">
       <c r="F55" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="G55" s="56">
         <v>-310</v>
@@ -9968,7 +10063,7 @@
     </row>
     <row r="56" spans="3:14" x14ac:dyDescent="0.25">
       <c r="F56" t="s">
-        <v>181</v>
+        <v>190</v>
       </c>
       <c r="G56" s="56">
         <v>-250</v>
@@ -9979,7 +10074,7 @@
     </row>
     <row r="57" spans="3:14" x14ac:dyDescent="0.25">
       <c r="F57" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="G57" s="56">
         <v>4690</v>
@@ -9990,7 +10085,7 @@
     </row>
     <row r="58" spans="3:14" x14ac:dyDescent="0.25">
       <c r="F58" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="G58" s="56">
         <v>-4440</v>
@@ -10001,7 +10096,7 @@
     </row>
     <row r="59" spans="3:14" x14ac:dyDescent="0.25">
       <c r="F59" t="s">
-        <v>182</v>
+        <v>191</v>
       </c>
       <c r="G59" s="56">
         <v>-4697</v>
@@ -10011,7 +10106,7 @@
     </row>
     <row r="60" spans="3:14" x14ac:dyDescent="0.25">
       <c r="F60" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
       <c r="G60" s="56">
         <v>-2500</v>
@@ -10021,7 +10116,7 @@
     </row>
     <row r="61" spans="3:14" x14ac:dyDescent="0.25">
       <c r="F61" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="G61" s="56">
         <v>-126</v>
@@ -10031,7 +10126,7 @@
     </row>
     <row r="62" spans="3:14" x14ac:dyDescent="0.25">
       <c r="F62" t="s">
-        <v>185</v>
+        <v>194</v>
       </c>
       <c r="G62" s="56">
         <v>4742</v>
@@ -10041,7 +10136,7 @@
     </row>
     <row r="63" spans="3:14" x14ac:dyDescent="0.25">
       <c r="F63" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="G63" s="56">
         <v>-410</v>
@@ -10056,7 +10151,7 @@
     </row>
     <row r="65" spans="2:9" x14ac:dyDescent="0.25">
       <c r="F65" t="s">
-        <v>186</v>
+        <v>195</v>
       </c>
       <c r="G65" s="56">
         <v>3320</v>
@@ -10066,7 +10161,7 @@
     </row>
     <row r="66" spans="2:9" x14ac:dyDescent="0.25">
       <c r="F66" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="G66" s="56">
         <v>4090</v>
@@ -10076,7 +10171,7 @@
     </row>
     <row r="67" spans="2:9" x14ac:dyDescent="0.25">
       <c r="F67" t="s">
-        <v>188</v>
+        <v>197</v>
       </c>
       <c r="G67" s="56">
         <v>-5688</v>
@@ -10086,7 +10181,7 @@
     </row>
     <row r="68" spans="2:9" x14ac:dyDescent="0.25">
       <c r="F68" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="G68" s="56">
         <v>-4433</v>
@@ -10096,7 +10191,7 @@
     </row>
     <row r="69" spans="2:9" x14ac:dyDescent="0.25">
       <c r="F69" t="s">
-        <v>189</v>
+        <v>198</v>
       </c>
       <c r="G69" s="56">
         <v>-250</v>
@@ -10108,7 +10203,7 @@
       <c r="C70" s="56"/>
       <c r="D70" s="56"/>
       <c r="F70" t="s">
-        <v>226</v>
+        <v>128</v>
       </c>
       <c r="G70" s="56">
         <v>-99</v>
@@ -10118,7 +10213,7 @@
     </row>
     <row r="71" spans="2:9" x14ac:dyDescent="0.25">
       <c r="F71" t="s">
-        <v>232</v>
+        <v>199</v>
       </c>
       <c r="G71" s="56">
         <v>320</v>
@@ -10128,7 +10223,7 @@
     </row>
     <row r="72" spans="2:9" x14ac:dyDescent="0.25">
       <c r="F72" t="s">
-        <v>233</v>
+        <v>200</v>
       </c>
       <c r="G72" s="56">
         <v>-1572</v>
@@ -10142,16 +10237,23 @@
       <c r="I73" s="56"/>
     </row>
     <row r="74" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="G74" s="56"/>
+      <c r="C74" s="56"/>
+      <c r="D74" s="56"/>
+      <c r="F74" t="s">
+        <v>159</v>
+      </c>
+      <c r="G74" s="56">
+        <v>4433</v>
+      </c>
       <c r="H74" s="56"/>
       <c r="I74" s="56"/>
     </row>
     <row r="75" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B75" t="s">
-        <v>150</v>
+        <v>201</v>
       </c>
       <c r="C75" s="56">
-        <v>4433</v>
+        <v>8000</v>
       </c>
       <c r="D75" s="56"/>
       <c r="G75" s="56"/>
@@ -10159,19 +10261,19 @@
       <c r="I75" s="56"/>
     </row>
     <row r="76" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B76" t="s">
-        <v>190</v>
-      </c>
-      <c r="C76" s="56">
-        <v>8000</v>
-      </c>
+      <c r="C76" s="56"/>
       <c r="D76" s="56"/>
       <c r="G76" s="56"/>
       <c r="H76" s="56"/>
       <c r="I76" s="56"/>
     </row>
     <row r="77" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C77" s="56"/>
+      <c r="B77" t="s">
+        <v>202</v>
+      </c>
+      <c r="C77" s="56">
+        <v>-50</v>
+      </c>
       <c r="D77" s="56"/>
       <c r="G77" s="56"/>
       <c r="H77" s="56"/>
@@ -10179,44 +10281,44 @@
     </row>
     <row r="78" spans="2:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B78" t="s">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="C78" s="56">
-        <v>-90</v>
-      </c>
-      <c r="D78" s="56"/>
+        <v>500</v>
+      </c>
+      <c r="D78" s="56">
+        <v>300</v>
+      </c>
       <c r="G78" s="56"/>
       <c r="H78" s="56"/>
       <c r="I78" s="56"/>
     </row>
     <row r="79" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B79" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="C79" s="56">
-        <v>1000</v>
-      </c>
-      <c r="D79" s="56">
-        <v>300</v>
-      </c>
+        <v>8000</v>
+      </c>
+      <c r="D79" s="56"/>
       <c r="G79" s="56"/>
       <c r="H79" s="56"/>
       <c r="I79" s="56"/>
     </row>
     <row r="80" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B80" t="s">
-        <v>193</v>
-      </c>
-      <c r="C80" s="56">
-        <v>8000</v>
-      </c>
+      <c r="C80" s="56"/>
       <c r="D80" s="56"/>
       <c r="G80" s="56"/>
       <c r="H80" s="56"/>
       <c r="I80" s="56"/>
     </row>
     <row r="81" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C81" s="56"/>
+      <c r="B81" t="s">
+        <v>202</v>
+      </c>
+      <c r="C81" s="56">
+        <v>-90</v>
+      </c>
       <c r="D81" s="56"/>
       <c r="G81" s="56"/>
       <c r="H81" s="56"/>
@@ -10224,88 +10326,88 @@
     </row>
     <row r="82" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B82" t="s">
-        <v>191</v>
+        <v>205</v>
       </c>
       <c r="C82" s="56">
-        <v>-90</v>
-      </c>
-      <c r="D82" s="56"/>
+        <v>2000</v>
+      </c>
+      <c r="D82" s="56">
+        <v>300</v>
+      </c>
       <c r="G82" s="56"/>
       <c r="H82" s="56"/>
       <c r="I82" s="56"/>
     </row>
     <row r="83" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B83" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="C83" s="56">
-        <v>2000</v>
-      </c>
-      <c r="D83" s="56">
-        <v>300</v>
-      </c>
+        <v>-12807</v>
+      </c>
+      <c r="D83" s="56"/>
       <c r="G83" s="56"/>
       <c r="H83" s="56"/>
       <c r="I83" s="56"/>
     </row>
     <row r="84" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B84" t="s">
-        <v>195</v>
-      </c>
-      <c r="C84" s="56">
-        <v>-12807</v>
-      </c>
+      <c r="C84" s="56"/>
       <c r="D84" s="56"/>
       <c r="G84" s="56"/>
       <c r="H84" s="56"/>
       <c r="I84" s="56"/>
     </row>
     <row r="85" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C85" s="56"/>
+      <c r="B85" t="s">
+        <v>207</v>
+      </c>
+      <c r="C85" s="56">
+        <v>5520</v>
+      </c>
       <c r="D85" s="56"/>
       <c r="G85" s="56"/>
       <c r="H85" s="56"/>
       <c r="I85" s="56"/>
     </row>
     <row r="86" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B86" t="s">
-        <v>196</v>
-      </c>
-      <c r="C86" s="56">
-        <v>5520</v>
-      </c>
+      <c r="C86" s="56"/>
       <c r="D86" s="56"/>
       <c r="G86" s="56"/>
       <c r="H86" s="56"/>
       <c r="I86" s="56"/>
     </row>
     <row r="87" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C87" s="56"/>
-      <c r="D87" s="56"/>
+      <c r="B87" t="s">
+        <v>208</v>
+      </c>
+      <c r="C87" s="56">
+        <v>2000</v>
+      </c>
+      <c r="D87" s="56">
+        <v>300</v>
+      </c>
       <c r="G87" s="56"/>
       <c r="H87" s="56"/>
       <c r="I87" s="56"/>
     </row>
     <row r="88" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B88" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="C88" s="56">
-        <v>2000</v>
-      </c>
-      <c r="D88" s="56">
-        <v>300</v>
-      </c>
+        <v>-90</v>
+      </c>
+      <c r="D88" s="56"/>
       <c r="G88" s="56"/>
       <c r="H88" s="56"/>
       <c r="I88" s="56"/>
     </row>
     <row r="89" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B89" t="s">
-        <v>191</v>
+        <v>209</v>
       </c>
       <c r="C89" s="56">
-        <v>-90</v>
+        <v>240</v>
       </c>
       <c r="D89" s="56"/>
       <c r="G89" s="56"/>
@@ -10313,44 +10415,44 @@
       <c r="I89" s="56"/>
     </row>
     <row r="90" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B90" t="s">
-        <v>198</v>
-      </c>
-      <c r="C90" s="56">
-        <v>240</v>
-      </c>
+      <c r="C90" s="56"/>
       <c r="D90" s="56"/>
       <c r="G90" s="56"/>
       <c r="H90" s="56"/>
       <c r="I90" s="56"/>
     </row>
     <row r="91" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C91" s="56"/>
-      <c r="D91" s="56"/>
+      <c r="B91" t="s">
+        <v>210</v>
+      </c>
+      <c r="C91" s="56">
+        <v>2000</v>
+      </c>
+      <c r="D91" s="56">
+        <v>300</v>
+      </c>
       <c r="G91" s="56"/>
       <c r="H91" s="56"/>
       <c r="I91" s="56"/>
     </row>
     <row r="92" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B92" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="C92" s="56">
-        <v>2000</v>
-      </c>
-      <c r="D92" s="56">
-        <v>300</v>
-      </c>
+        <v>-50</v>
+      </c>
+      <c r="D92" s="56"/>
       <c r="G92" s="56"/>
       <c r="H92" s="56"/>
       <c r="I92" s="56"/>
     </row>
     <row r="93" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B93" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
       <c r="C93" s="56">
-        <v>-50</v>
+        <v>300</v>
       </c>
       <c r="D93" s="56"/>
       <c r="G93" s="56"/>
@@ -10358,44 +10460,44 @@
       <c r="I93" s="56"/>
     </row>
     <row r="94" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B94" t="s">
-        <v>201</v>
-      </c>
-      <c r="C94" s="56">
-        <v>300</v>
-      </c>
+      <c r="C94" s="56"/>
       <c r="D94" s="56"/>
       <c r="G94" s="56"/>
       <c r="H94" s="56"/>
       <c r="I94" s="56"/>
     </row>
     <row r="95" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C95" s="56"/>
-      <c r="D95" s="56"/>
+      <c r="B95" t="s">
+        <v>213</v>
+      </c>
+      <c r="C95" s="56">
+        <v>2000</v>
+      </c>
+      <c r="D95" s="56">
+        <v>300</v>
+      </c>
       <c r="G95" s="56"/>
       <c r="H95" s="56"/>
       <c r="I95" s="56"/>
     </row>
     <row r="96" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B96" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="C96" s="56">
-        <v>2000</v>
-      </c>
-      <c r="D96" s="56">
-        <v>300</v>
-      </c>
+        <v>8000</v>
+      </c>
+      <c r="D96" s="56"/>
       <c r="G96" s="56"/>
       <c r="H96" s="56"/>
       <c r="I96" s="56"/>
     </row>
     <row r="97" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B97" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="C97" s="56">
-        <v>8000</v>
+        <v>4180</v>
       </c>
       <c r="D97" s="56"/>
       <c r="G97" s="56"/>
@@ -10403,27 +10505,29 @@
       <c r="I97" s="56"/>
     </row>
     <row r="98" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B98" t="s">
-        <v>204</v>
-      </c>
-      <c r="C98" s="56">
-        <v>4180</v>
-      </c>
+      <c r="C98" s="56"/>
       <c r="D98" s="56"/>
       <c r="G98" s="56"/>
       <c r="H98" s="56"/>
       <c r="I98" s="56"/>
     </row>
     <row r="99" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C99" s="56"/>
-      <c r="D99" s="56"/>
+      <c r="B99" t="s">
+        <v>216</v>
+      </c>
+      <c r="C99" s="56">
+        <v>2000</v>
+      </c>
+      <c r="D99" s="56">
+        <v>300</v>
+      </c>
       <c r="G99" s="56"/>
       <c r="H99" s="56"/>
       <c r="I99" s="56"/>
     </row>
     <row r="100" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B100" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="C100" s="56">
         <v>2000</v>
@@ -10437,7 +10541,7 @@
     </row>
     <row r="101" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B101" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="C101" s="56">
         <v>2000</v>
@@ -10450,48 +10554,48 @@
       <c r="I101" s="56"/>
     </row>
     <row r="102" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B102" t="s">
-        <v>207</v>
-      </c>
-      <c r="C102" s="56">
-        <v>2000</v>
-      </c>
-      <c r="D102" s="56">
-        <v>300</v>
-      </c>
+      <c r="C102" s="56"/>
+      <c r="D102" s="56"/>
       <c r="G102" s="56"/>
       <c r="H102" s="56"/>
       <c r="I102" s="56"/>
     </row>
     <row r="103" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C103" s="56"/>
+      <c r="B103" t="s">
+        <v>219</v>
+      </c>
+      <c r="C103" s="56">
+        <v>-20000</v>
+      </c>
       <c r="D103" s="56"/>
       <c r="G103" s="56"/>
       <c r="H103" s="56"/>
       <c r="I103" s="56"/>
     </row>
     <row r="104" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B104" t="s">
-        <v>208</v>
-      </c>
-      <c r="C104" s="56">
-        <v>-20000</v>
-      </c>
+      <c r="C104" s="56"/>
       <c r="D104" s="56"/>
       <c r="G104" s="56"/>
       <c r="H104" s="56"/>
       <c r="I104" s="56"/>
     </row>
     <row r="105" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="C105" s="56"/>
-      <c r="D105" s="56"/>
+      <c r="B105" t="s">
+        <v>220</v>
+      </c>
+      <c r="C105" s="56">
+        <v>2000</v>
+      </c>
+      <c r="D105" s="56">
+        <v>300</v>
+      </c>
       <c r="G105" s="56"/>
       <c r="H105" s="56"/>
       <c r="I105" s="56"/>
     </row>
     <row r="106" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B106" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="C106" s="56">
         <v>2000</v>
@@ -10505,33 +10609,33 @@
     </row>
     <row r="107" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B107" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="C107" s="56">
-        <v>2000</v>
-      </c>
-      <c r="D107" s="56">
-        <v>300</v>
-      </c>
+        <v>8000</v>
+      </c>
+      <c r="D107" s="56"/>
       <c r="G107" s="56"/>
       <c r="H107" s="56"/>
       <c r="I107" s="56"/>
     </row>
     <row r="108" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B108" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
       <c r="C108" s="56">
-        <v>8000</v>
-      </c>
-      <c r="D108" s="56"/>
+        <v>2000</v>
+      </c>
+      <c r="D108" s="56">
+        <v>300</v>
+      </c>
       <c r="G108" s="56"/>
       <c r="H108" s="56"/>
       <c r="I108" s="56"/>
     </row>
     <row r="109" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B109" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="C109" s="56">
         <v>2000</v>
@@ -10544,15 +10648,6 @@
       <c r="I109" s="56"/>
     </row>
     <row r="110" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B110" t="s">
-        <v>213</v>
-      </c>
-      <c r="C110" s="56">
-        <v>2000</v>
-      </c>
-      <c r="D110" s="56">
-        <v>300</v>
-      </c>
       <c r="G110" s="56"/>
       <c r="H110" s="56"/>
       <c r="I110" s="56"/>
@@ -11757,43 +11852,43 @@
     <mergeCell ref="M3:M4"/>
   </mergeCells>
   <phoneticPr fontId="15" type="noConversion"/>
-  <conditionalFormatting sqref="B5:C5 C70:D70 C75:D110">
-    <cfRule type="cellIs" dxfId="9" priority="67" operator="greaterThan">
+  <conditionalFormatting sqref="B5:C5 C70:D70 C74:D109">
+    <cfRule type="cellIs" dxfId="9" priority="85" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="68" operator="lessThan">
+    <cfRule type="cellIs" dxfId="8" priority="86" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C14:D52">
-    <cfRule type="cellIs" dxfId="7" priority="61" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="7" priority="79" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="62" operator="lessThan">
+    <cfRule type="cellIs" dxfId="6" priority="80" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G120:G1048576">
-    <cfRule type="cellIs" dxfId="5" priority="63" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="81" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="64" operator="lessThan">
+    <cfRule type="cellIs" dxfId="4" priority="82" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G14:I119">
-    <cfRule type="cellIs" dxfId="3" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="4" operator="lessThan">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H120:I266">
-    <cfRule type="cellIs" dxfId="1" priority="65" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="83" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="66" operator="lessThan">
+    <cfRule type="cellIs" dxfId="0" priority="84" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11815,13 +11910,13 @@
   <sheetData>
     <row r="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B1" s="65" t="s">
-        <v>214</v>
+        <v>225</v>
       </c>
       <c r="C1" s="66" t="s">
-        <v>215</v>
+        <v>226</v>
       </c>
       <c r="D1" s="65" t="s">
-        <v>216</v>
+        <v>227</v>
       </c>
     </row>
     <row r="2" spans="2:4" x14ac:dyDescent="0.25">
@@ -11829,77 +11924,77 @@
         <v>22</v>
       </c>
       <c r="C2" s="40" t="s">
-        <v>217</v>
+        <v>228</v>
       </c>
       <c r="D2" s="57"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="57" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="C3" s="40" t="s">
-        <v>217</v>
+        <v>228</v>
       </c>
       <c r="D3" s="57"/>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" s="57" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="C4" s="40" t="s">
-        <v>218</v>
+        <v>229</v>
       </c>
       <c r="D4" s="57"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B5" s="57" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="C5" s="40" t="s">
-        <v>217</v>
+        <v>228</v>
       </c>
       <c r="D5" s="57"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" s="57" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="C6" s="40" t="s">
-        <v>218</v>
+        <v>229</v>
       </c>
       <c r="D6" s="57"/>
     </row>
     <row r="7" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B7" s="57" t="s">
-        <v>219</v>
+        <v>230</v>
       </c>
       <c r="C7" s="40" t="s">
-        <v>218</v>
+        <v>229</v>
       </c>
       <c r="D7" s="57"/>
     </row>
     <row r="8" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B8" s="57" t="s">
-        <v>220</v>
+        <v>231</v>
       </c>
       <c r="C8" s="40" t="s">
-        <v>218</v>
+        <v>229</v>
       </c>
       <c r="D8" s="57"/>
     </row>
     <row r="9" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B9" s="57" t="s">
-        <v>221</v>
+        <v>232</v>
       </c>
       <c r="C9" s="40"/>
       <c r="D9" s="57"/>
     </row>
     <row r="10" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B10" s="57" t="s">
-        <v>222</v>
+        <v>233</v>
       </c>
       <c r="C10" s="40" t="s">
-        <v>217</v>
+        <v>228</v>
       </c>
       <c r="D10" s="57"/>
     </row>

</xml_diff>